<commit_message>
Updated IDN_grids_kan model - 2026-05-06 22:30
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2E9DF7A-B1AA-4C1E-8855-53BF818222EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{966D5566-EB2A-4D62-A2E4-74655289BF26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AED5CFC-E4F3-4B66-BDF3-D607C62E9241}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8BC3C5-8C6B-4A33-9F47-EF33A9A46234}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B70617-5DBA-4C59-BDF2-D5464F062DC1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3AA9186-FC6C-4C61-B901-A94650532846}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IDN_grids_kan model - 2026-05-06 23:04
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{966D5566-EB2A-4D62-A2E4-74655289BF26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1116342-48AC-4175-AEFC-707E4A945B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4321,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8BC3C5-8C6B-4A33-9F47-EF33A9A46234}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCC469A4-E50E-47CA-BFDB-C4D29AE44E4C}">
   <dimension ref="B9:H263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27634,7 +27634,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3AA9186-FC6C-4C61-B901-A94650532846}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6D3BF2C-E68D-49AA-BEA7-78FACB9109D7}">
   <dimension ref="B9:L263"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>